<commit_message>
Tableau de bord provincial (lecture seule) — mise à jour du 15/10/2026 22:38
</commit_message>
<xml_diff>
--- a/nord-kivu/sortie/zs/Alimbongo/Tableaux_ZS_Alimbongo_20261014.xlsx
+++ b/nord-kivu/sortie/zs/Alimbongo/Tableaux_ZS_Alimbongo_20261014.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bulletin des aires'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bulletin des aires'!$A$1:$P$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cas'!$A$1:$S$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -452,11 +452,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -585,8 +585,32 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kitsumbiro</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Non touchée</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:P3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>